<commit_message>
Bloque 5: leer circuitos desde Excel con openpyxl
</commit_message>
<xml_diff>
--- a/circuitos.xlsx
+++ b/circuitos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user007\Documents\motor-calculo-bt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5CB1280-86E7-4317-98A4-544685F17296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB48BD12-A0D3-4C70-A175-FDAE56161638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="30">
   <si>
     <t>Nombre</t>
   </si>
@@ -90,6 +90,42 @@
   </si>
   <si>
     <t>0.90</t>
+  </si>
+  <si>
+    <t>temp_amb</t>
+  </si>
+  <si>
+    <t>Iluminacion HUB</t>
+  </si>
+  <si>
+    <t>Sistema</t>
+  </si>
+  <si>
+    <t>Paralelos</t>
+  </si>
+  <si>
+    <t>3F</t>
+  </si>
+  <si>
+    <t>1F</t>
+  </si>
+  <si>
+    <t>Tomacorriente Oficina</t>
+  </si>
+  <si>
+    <t>12AWG</t>
+  </si>
+  <si>
+    <t>10AWG</t>
+  </si>
+  <si>
+    <t>1.00</t>
+  </si>
+  <si>
+    <t>Mini Split 1-A</t>
+  </si>
+  <si>
+    <t>2F</t>
   </si>
 </sst>
 </file>
@@ -461,146 +497,297 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA913B4-B8F6-49BC-B857-96228659B976}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
         <v>12</v>
       </c>
-      <c r="C2">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
         <v>63</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-      <c r="C3">
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
         <v>63</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="C4">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
         <v>63</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="E4">
+      <c r="G4">
         <v>80</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="C5">
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
         <v>63</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>17</v>
       </c>
-      <c r="E5">
+      <c r="G5">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
         <v>14</v>
       </c>
-      <c r="C6">
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
         <v>63</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>17</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
       <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
         <v>15</v>
       </c>
-      <c r="C7">
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
         <v>500</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>17</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
       <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
         <v>15</v>
       </c>
-      <c r="C8">
+      <c r="D8">
+        <v>4</v>
+      </c>
+      <c r="E8">
         <v>500</v>
       </c>
-      <c r="D8" t="s">
+      <c r="F8" t="s">
         <v>17</v>
       </c>
-      <c r="E8">
+      <c r="G8">
         <v>15</v>
+      </c>
+      <c r="H8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9">
+        <v>80</v>
+      </c>
+      <c r="H9">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+      <c r="F10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10">
+        <v>25</v>
+      </c>
+      <c r="H10">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11">
+        <v>15</v>
+      </c>
+      <c r="H11">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Etapa 3 M1: leer_transformador_excel() desde hoja Excel
</commit_message>
<xml_diff>
--- a/circuitos.xlsx
+++ b/circuitos.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user007\Documents\motor-calculo-bt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22876F1B-3A5A-4EC3-BAAB-7F71A4B33E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E18B93C0-78BE-457F-BF1E-452678EFE3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" activeTab="1" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="circuitos" sheetId="1" r:id="rId1"/>
+    <sheet name="Transformador" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="42">
   <si>
     <t>Nombre</t>
   </si>
@@ -126,6 +127,42 @@
   </si>
   <si>
     <t>2F</t>
+  </si>
+  <si>
+    <t>campo</t>
+  </si>
+  <si>
+    <t>valor</t>
+  </si>
+  <si>
+    <t>nombre</t>
+  </si>
+  <si>
+    <t>Trasformador N°1</t>
+  </si>
+  <si>
+    <t>modo</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>KVA</t>
+  </si>
+  <si>
+    <t>Vn_BT</t>
+  </si>
+  <si>
+    <t>Ucc_pct</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>conexión</t>
+  </si>
+  <si>
+    <t>Dyn11</t>
   </si>
 </sst>
 </file>
@@ -793,4 +830,73 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC923F8D-0FAA-4C09-BC0E-B1B2A5D10AEB}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Etapa 3 M3: protecciones.py + 15 tests nuevos (54 total)
</commit_message>
<xml_diff>
--- a/circuitos.xlsx
+++ b/circuitos.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user007\Documents\motor-calculo-bt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E18B93C0-78BE-457F-BF1E-452678EFE3D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC40798B-B76E-481E-8929-D6DF8CA34421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" activeTab="1" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
   </bookViews>
   <sheets>
     <sheet name="circuitos" sheetId="1" r:id="rId1"/>
     <sheet name="Transformador" sheetId="2" r:id="rId2"/>
+    <sheet name="Protecciones" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="47">
   <si>
     <t>Nombre</t>
   </si>
@@ -60,9 +61,6 @@
     <t>CRAC Unit 1-B</t>
   </si>
   <si>
-    <t>Antenna Panel campo</t>
-  </si>
-  <si>
     <t>STS Panel BUS A</t>
   </si>
   <si>
@@ -163,6 +161,24 @@
   </si>
   <si>
     <t>Dyn11</t>
+  </si>
+  <si>
+    <t>Curva</t>
+  </si>
+  <si>
+    <t>In_A</t>
+  </si>
+  <si>
+    <t>Poder_Corte_KA</t>
+  </si>
+  <si>
+    <t>TM</t>
+  </si>
+  <si>
+    <t>Antena Panel campo</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
@@ -546,13 +562,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
@@ -564,7 +580,7 @@
         <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -572,10 +588,10 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -584,7 +600,7 @@
         <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G2">
         <v>10</v>
@@ -598,10 +614,10 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -610,7 +626,7 @@
         <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G3">
         <v>10</v>
@@ -621,13 +637,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -636,7 +652,7 @@
         <v>63</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G4">
         <v>80</v>
@@ -647,13 +663,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -662,7 +678,7 @@
         <v>63</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G5">
         <v>20</v>
@@ -673,13 +689,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -688,7 +704,7 @@
         <v>63</v>
       </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G6">
         <v>20</v>
@@ -699,13 +715,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -714,7 +730,7 @@
         <v>500</v>
       </c>
       <c r="F7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G7">
         <v>15</v>
@@ -725,13 +741,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -740,7 +756,7 @@
         <v>500</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8">
         <v>15</v>
@@ -751,13 +767,13 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -766,7 +782,7 @@
         <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G9">
         <v>80</v>
@@ -777,13 +793,13 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -792,7 +808,7 @@
         <v>20</v>
       </c>
       <c r="F10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G10">
         <v>25</v>
@@ -803,13 +819,13 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
         <v>28</v>
       </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -818,7 +834,7 @@
         <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G11">
         <v>15</v>
@@ -842,31 +858,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
         <v>30</v>
-      </c>
-      <c r="B1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
         <v>34</v>
-      </c>
-      <c r="B3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4">
         <v>1000</v>
@@ -874,7 +890,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5">
         <v>380</v>
@@ -882,18 +898,186 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
         <v>38</v>
-      </c>
-      <c r="B6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
         <v>40</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D85B9E58-1743-4BDF-B358-88BA0F565778}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2">
+        <v>200</v>
+      </c>
+      <c r="D2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3">
+        <v>200</v>
+      </c>
+      <c r="D3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4">
+        <v>63</v>
+      </c>
+      <c r="D4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5">
+        <v>160</v>
+      </c>
+      <c r="D5">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6">
+        <v>160</v>
+      </c>
+      <c r="D6">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>46</v>
+      </c>
+      <c r="C7">
+        <v>400</v>
+      </c>
+      <c r="D7">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8">
+        <v>400</v>
+      </c>
+      <c r="D8">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9">
+        <v>16</v>
+      </c>
+      <c r="D9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10">
+        <v>25</v>
+      </c>
+      <c r="D10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11">
+        <v>16</v>
+      </c>
+      <c r="D11">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Etapa 3 M4: balance.py + lectura Excel + 6 tests nuevos (60 total)
</commit_message>
<xml_diff>
--- a/circuitos.xlsx
+++ b/circuitos.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user007\Documents\motor-calculo-bt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC40798B-B76E-481E-8929-D6DF8CA34421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5207376-E530-4F73-A4FB-7EF27D197427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" firstSheet="3" activeTab="3" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
   </bookViews>
   <sheets>
     <sheet name="circuitos" sheetId="1" r:id="rId1"/>
     <sheet name="Transformador" sheetId="2" r:id="rId2"/>
     <sheet name="Protecciones" sheetId="3" r:id="rId3"/>
+    <sheet name="Balance" sheetId="4" r:id="rId4"/>
+    <sheet name="tableros" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="59">
   <si>
     <t>Nombre</t>
   </si>
@@ -179,6 +181,42 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>Tablero</t>
+  </si>
+  <si>
+    <t>MDP</t>
+  </si>
+  <si>
+    <t>Fase</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>Tipo_carga</t>
+  </si>
+  <si>
+    <t>HVAC</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>UPS</t>
+  </si>
+  <si>
+    <t>Iluminacion</t>
+  </si>
+  <si>
+    <t>Tomacorriente</t>
+  </si>
+  <si>
+    <t>Capacidad_KVA</t>
   </si>
 </sst>
 </file>
@@ -1083,4 +1121,201 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{309AEC8C-FC61-41D6-9257-207B22A2FB81}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E3CA68-C546-414F-B821-889E69738B76}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2">
+        <v>1000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
M4.5: perfiles + validación + modo híbrido + bloqueo selector
</commit_message>
<xml_diff>
--- a/circuitos.xlsx
+++ b/circuitos.xlsx
@@ -2,52 +2,142 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user007\Documents\motor-calculo-bt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5207376-E530-4F73-A4FB-7EF27D197427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28240D7A-8826-41B9-80BF-52A4C56F8385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" firstSheet="3" activeTab="3" xr2:uid="{B1CA57BF-FAED-4221-8BEA-445E7669A704}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="circuitos" sheetId="1" r:id="rId1"/>
-    <sheet name="Transformador" sheetId="2" r:id="rId2"/>
-    <sheet name="Protecciones" sheetId="3" r:id="rId3"/>
-    <sheet name="Balance" sheetId="4" r:id="rId4"/>
-    <sheet name="tableros" sheetId="5" r:id="rId5"/>
+    <sheet name="perfil" sheetId="1" r:id="rId1"/>
+    <sheet name="circuitos" sheetId="2" r:id="rId2"/>
+    <sheet name="Transformador" sheetId="3" r:id="rId3"/>
+    <sheet name="Protecciones" sheetId="4" r:id="rId4"/>
+    <sheet name="Balance" sheetId="5" r:id="rId5"/>
+    <sheet name="tableros" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="78">
   <si>
     <t>Nombre</t>
   </si>
   <si>
+    <t>Curva</t>
+  </si>
+  <si>
+    <t>In_A</t>
+  </si>
+  <si>
+    <t>Poder_Corte_KA</t>
+  </si>
+  <si>
+    <t>CRAC Unit 1-A</t>
+  </si>
+  <si>
+    <t>TM</t>
+  </si>
+  <si>
+    <t>CRAC Unit 1-B</t>
+  </si>
+  <si>
+    <t>Antena Panel campo</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>STS Panel BUS A</t>
+  </si>
+  <si>
+    <t>STS Panel BUS B</t>
+  </si>
+  <si>
+    <t>Alimentacion UPS 1</t>
+  </si>
+  <si>
+    <t>Alimentacion UPS 2</t>
+  </si>
+  <si>
+    <t>Iluminacion HUB</t>
+  </si>
+  <si>
+    <t>Tomacorriente Oficina</t>
+  </si>
+  <si>
+    <t>Mini Split 1-A</t>
+  </si>
+  <si>
+    <t>PERFIL DE PROYECTO — Motor de Cálculo BT</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>perfil</t>
+  </si>
+  <si>
+    <t>industrial</t>
+  </si>
+  <si>
+    <t>Tipo de proyecto: domestico / comercial / industrial</t>
+  </si>
+  <si>
+    <t>nombre_proyecto</t>
+  </si>
+  <si>
+    <t>LEO-ARICA</t>
+  </si>
+  <si>
+    <t>Nombre del proyecto (se usa en el reporte)</t>
+  </si>
+  <si>
+    <t>usar_transformador</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>¿Incluir cálculo de transformador e Icc? si / no</t>
+  </si>
+  <si>
+    <t>usar_protecciones</t>
+  </si>
+  <si>
+    <t>¿Incluir verificación de protecciones? si / no</t>
+  </si>
+  <si>
+    <t>usar_balance</t>
+  </si>
+  <si>
+    <t>¿Incluir balance de carga por tablero? si / no</t>
+  </si>
+  <si>
+    <t>⚡  Usa los desplegables en la columna B para configurar el perfil. La herramienta detectará la configuración automáticamente al cargar este archivo.</t>
+  </si>
+  <si>
+    <t>Sistema</t>
+  </si>
+  <si>
     <t>Conductor</t>
   </si>
   <si>
+    <t>Paralelos</t>
+  </si>
+  <si>
     <t>I_diseno</t>
   </si>
   <si>
@@ -57,75 +147,42 @@
     <t>L_m</t>
   </si>
   <si>
-    <t>CRAC Unit 1-A</t>
-  </si>
-  <si>
-    <t>CRAC Unit 1-B</t>
-  </si>
-  <si>
-    <t>STS Panel BUS A</t>
-  </si>
-  <si>
-    <t>STS Panel BUS B</t>
-  </si>
-  <si>
-    <t>Alimentacion UPS 1</t>
-  </si>
-  <si>
-    <t>Alimentacion UPS 2</t>
+    <t>temp_amb</t>
+  </si>
+  <si>
+    <t>3F</t>
   </si>
   <si>
     <t>6AWG</t>
   </si>
   <si>
+    <t>0.85</t>
+  </si>
+  <si>
     <t>2AWG</t>
   </si>
   <si>
     <t>1/0AWG</t>
   </si>
   <si>
+    <t>0.90</t>
+  </si>
+  <si>
     <t>400MCM</t>
   </si>
   <si>
-    <t>0.85</t>
-  </si>
-  <si>
-    <t>0.90</t>
-  </si>
-  <si>
-    <t>temp_amb</t>
-  </si>
-  <si>
-    <t>Iluminacion HUB</t>
-  </si>
-  <si>
-    <t>Sistema</t>
-  </si>
-  <si>
-    <t>Paralelos</t>
-  </si>
-  <si>
-    <t>3F</t>
-  </si>
-  <si>
     <t>1F</t>
   </si>
   <si>
-    <t>Tomacorriente Oficina</t>
-  </si>
-  <si>
     <t>12AWG</t>
   </si>
   <si>
+    <t>1.00</t>
+  </si>
+  <si>
     <t>10AWG</t>
   </si>
   <si>
-    <t>1.00</t>
-  </si>
-  <si>
-    <t>Mini Split 1-A</t>
-  </si>
-  <si>
     <t>2F</t>
   </si>
   <si>
@@ -165,48 +222,30 @@
     <t>Dyn11</t>
   </si>
   <si>
-    <t>Curva</t>
-  </si>
-  <si>
-    <t>In_A</t>
-  </si>
-  <si>
-    <t>Poder_Corte_KA</t>
-  </si>
-  <si>
-    <t>TM</t>
-  </si>
-  <si>
-    <t>Antena Panel campo</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>Tablero</t>
   </si>
   <si>
+    <t>Fase</t>
+  </si>
+  <si>
+    <t>Tipo_carga</t>
+  </si>
+  <si>
     <t>MDP</t>
   </si>
   <si>
-    <t>Fase</t>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>HVAC</t>
+  </si>
+  <si>
+    <t>L2</t>
   </si>
   <si>
     <t>L3</t>
   </si>
   <si>
-    <t>Tipo_carga</t>
-  </si>
-  <si>
-    <t>HVAC</t>
-  </si>
-  <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>L2</t>
-  </si>
-  <si>
     <t>UPS</t>
   </si>
   <si>
@@ -217,13 +256,16 @@
   </si>
   <si>
     <t>Capacidad_KVA</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,16 +273,81 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF8888AA"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF5E81F4"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF666688"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF444466"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6E4F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2A2A3E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E1E2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEEFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -248,12 +355,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,7 +728,114 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA913B4-B8F6-49BC-B857-96228659B976}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A9:C9"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Perfil inválido" error="Selecciona: domestico, comercial o industrial" sqref="B3" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>"domestico,comercial,industrial"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Selecciona: si o no" sqref="B5:B7" xr:uid="{00000000-0002-0000-0000-000001000000}">
+      <formula1>"si,no"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -600,36 +848,36 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E1" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="F1" t="s">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="G1" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -638,7 +886,7 @@
         <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="G2">
         <v>10</v>
@@ -652,10 +900,10 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -664,7 +912,7 @@
         <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="G3">
         <v>10</v>
@@ -675,13 +923,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -690,7 +938,7 @@
         <v>63</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="G4">
         <v>80</v>
@@ -701,13 +949,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -716,7 +964,7 @@
         <v>63</v>
       </c>
       <c r="F5" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G5">
         <v>20</v>
@@ -727,13 +975,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -742,7 +990,7 @@
         <v>63</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G6">
         <v>20</v>
@@ -753,13 +1001,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -768,7 +1016,7 @@
         <v>500</v>
       </c>
       <c r="F7" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G7">
         <v>15</v>
@@ -779,13 +1027,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="D8">
         <v>4</v>
@@ -794,7 +1042,7 @@
         <v>500</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G8">
         <v>15</v>
@@ -805,13 +1053,13 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -820,7 +1068,7 @@
         <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="G9">
         <v>80</v>
@@ -831,13 +1079,13 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -846,7 +1094,7 @@
         <v>20</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="G10">
         <v>25</v>
@@ -857,13 +1105,13 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -872,7 +1120,7 @@
         <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G11">
         <v>15</v>
@@ -886,8 +1134,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC923F8D-0FAA-4C09-BC0E-B1B2A5D10AEB}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -896,31 +1144,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="B4">
         <v>1000</v>
@@ -928,7 +1176,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="B5">
         <v>380</v>
@@ -936,18 +1184,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -955,8 +1203,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D85B9E58-1743-4BDF-B358-88BA0F565778}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -969,21 +1217,21 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>43</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
       </c>
       <c r="C2">
         <v>200</v>
@@ -997,7 +1245,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>200</v>
@@ -1008,10 +1256,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>63</v>
@@ -1022,10 +1270,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>160</v>
@@ -1036,10 +1284,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>46</v>
       </c>
       <c r="C6">
         <v>160</v>
@@ -1050,10 +1298,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C7">
         <v>400</v>
@@ -1064,10 +1312,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C8">
         <v>400</v>
@@ -1078,10 +1326,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C9">
         <v>16</v>
@@ -1092,10 +1340,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C10">
         <v>25</v>
@@ -1106,10 +1354,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C11">
         <v>16</v>
@@ -1123,8 +1371,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{309AEC8C-FC61-41D6-9257-207B22A2FB81}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1137,27 +1385,27 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="C1" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1165,125 +1413,125 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1291,8 +1539,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E3CA68-C546-414F-B821-889E69738B76}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1304,12 +1552,12 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="B2">
         <v>1000</v>

</xml_diff>

<commit_message>
M7 Fase 1: coordinacion.py + leer_cadena_excel + hoja cadena Excel + integración main + 90 tests
</commit_message>
<xml_diff>
--- a/circuitos.xlsx
+++ b/circuitos.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tableros" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demanda" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cadena" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -94,8 +95,13 @@
       <color rgb="FF444466"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF5E81F4"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -132,6 +138,11 @@
         <fgColor rgb="FFEEEEFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF252535"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -166,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -205,6 +216,13 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -719,7 +737,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="30" customHeight="1" s="6">
       <c r="A9" s="7" t="inlineStr">
         <is>
@@ -1965,4 +1982,435 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="6" min="1" max="1"/>
+    <col width="14" customWidth="1" style="6" min="2" max="2"/>
+    <col width="16" customWidth="1" style="6" min="3" max="3"/>
+    <col width="7" customWidth="1" style="6" min="4" max="4"/>
+    <col width="9" customWidth="1" style="6" min="5" max="5"/>
+    <col width="9" customWidth="1" style="6" min="6" max="6"/>
+    <col width="8" customWidth="1" style="6" min="7" max="7"/>
+    <col width="9" customWidth="1" style="6" min="8" max="8"/>
+    <col width="8" customWidth="1" style="6" min="9" max="9"/>
+    <col width="8" customWidth="1" style="6" min="10" max="10"/>
+    <col width="12" customWidth="1" style="6" min="11" max="11"/>
+    <col width="18" customWidth="1" style="6" min="12" max="12"/>
+    <col width="9" customWidth="1" style="6" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="6">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>CADENA DE PROTECCIONES — Motor de Cálculo BT M7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" s="6">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>designacion</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>circuito_ref</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>nivel</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>In_A</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>curva</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>Ir_xIn</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>Isd_xIr</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>tsd_s</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>Ii_xIn</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>modo</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>upstream</t>
+        </is>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>Icc_kA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>G0A_3WA1600</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>IA_5.1B</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>BTDP_5.1</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="14" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>ETU600</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K3" s="14" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="L3" s="14" t="inlineStr"/>
+      <c r="M3" s="14" t="n">
+        <v>30.39</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>G1A_3VA630</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>IA_11.1B</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>BTDP_11.1</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>630</v>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>ETU320</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H4" s="15" t="inlineStr"/>
+      <c r="I4" s="15" t="inlineStr"/>
+      <c r="J4" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>G0A_3WA1600</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="n">
+        <v>10.77</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>C1A_3VA160</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>IA_12.1A</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>BTSD_12.1</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>160</v>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>ETU320</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H5" s="14" t="inlineStr"/>
+      <c r="I5" s="14" t="inlineStr"/>
+      <c r="J5" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="L5" s="14" t="inlineStr">
+        <is>
+          <t>G1A_3VA630</t>
+        </is>
+      </c>
+      <c r="M5" s="14" t="n">
+        <v>6.22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>C2A_5SY32</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>IA_12.2A</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Antena</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="15" t="inlineStr"/>
+      <c r="I6" s="15" t="inlineStr"/>
+      <c r="J6" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>C1A_3VA160</t>
+        </is>
+      </c>
+      <c r="M6" s="15" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>G0B_3WA1000</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>IA_4.1B</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>BTDP_4.1</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>ETU600</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>generador</t>
+        </is>
+      </c>
+      <c r="L7" s="14" t="inlineStr"/>
+      <c r="M7" s="14" t="n">
+        <v>9.08</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>C1B_3VA200</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>IA_18.2A</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>BTSD_18.1</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>TM</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H8" s="15" t="inlineStr"/>
+      <c r="I8" s="15" t="inlineStr"/>
+      <c r="J8" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>generador</t>
+        </is>
+      </c>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>G0B_3WA1000</t>
+        </is>
+      </c>
+      <c r="M8" s="15" t="n">
+        <v>2.06</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr"/>
+      <c r="B9" s="16" t="inlineStr"/>
+      <c r="C9" s="16" t="inlineStr"/>
+      <c r="D9" s="16" t="inlineStr"/>
+      <c r="E9" s="16" t="inlineStr"/>
+      <c r="F9" s="16" t="inlineStr"/>
+      <c r="G9" s="16" t="inlineStr"/>
+      <c r="H9" s="16" t="inlineStr"/>
+      <c r="I9" s="16" t="inlineStr"/>
+      <c r="J9" s="16" t="inlineStr"/>
+      <c r="K9" s="16" t="inlineStr"/>
+      <c r="L9" s="16" t="inlineStr"/>
+      <c r="M9" s="16" t="inlineStr"/>
+    </row>
+    <row r="11" ht="36" customHeight="1" s="6">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>⚡  M7 usa esta hoja para verificar selectividad TCC y cumplimiento IEC 60364-4-41. Curva ETU: región térmica (Ir &lt; Icc &lt; Isd) no modelada → usar SIMARIS. Orden: nivel 0 = cabecera, niveles crecientes aguas abajo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="F3:F100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Curva inválida" error="Selecciona: ETU600, ETU320, TM, C, D o B" type="list">
+      <formula1>"ETU600,ETU320,TM,C,D,B"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K3:K100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Modo inválido" error="Selecciona: red, generador o acople" type="list">
+      <formula1>"red,generador,acople"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Petitorio v1: persistencia, dashboard, contrato salida EPC
</commit_message>
<xml_diff>
--- a/circuitos.xlsx
+++ b/circuitos.xlsx
@@ -787,7 +787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="20.42578125" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -835,6 +835,11 @@
           <t>temp_amb</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>norma</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -869,6 +874,11 @@
       <c r="H2" t="n">
         <v>30</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -903,6 +913,11 @@
       <c r="H3" t="n">
         <v>30</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -937,6 +952,11 @@
       <c r="H4" t="n">
         <v>35</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -971,6 +991,11 @@
       <c r="H5" t="n">
         <v>30</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1005,6 +1030,11 @@
       <c r="H6" t="n">
         <v>30</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1039,6 +1069,11 @@
       <c r="H7" t="n">
         <v>30</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1073,6 +1108,11 @@
       <c r="H8" t="n">
         <v>30</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1107,6 +1147,11 @@
       <c r="H9" t="n">
         <v>35</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1141,6 +1186,11 @@
       <c r="H10" t="n">
         <v>30</v>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1174,6 +1224,11 @@
       </c>
       <c r="H11" t="n">
         <v>30</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>AWG</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>